<commit_message>
data modelling for user given data, AI tool compnay data, output data and other data for system design and UI design
</commit_message>
<xml_diff>
--- a/pricing-comparison.xlsx
+++ b/pricing-comparison.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\projects\leak-AI-cost-detector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5846A1F3-2DD0-4354-A4A3-45020E0F5199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4834485-6CD0-4336-A480-26750146DB09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$K$1:$K$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$K$1:$K$140</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="148">
   <si>
     <t>cursor</t>
   </si>
@@ -457,19 +457,74 @@
   </si>
   <si>
     <t>max output tokens</t>
+  </si>
+  <si>
+    <t>chatgpt Business Codex</t>
+  </si>
+  <si>
+    <t>chatgpt credits plan</t>
+  </si>
+  <si>
+    <t>Gemini google Workspace 
+(for business)</t>
+  </si>
+  <si>
+    <t>Gemini Enterprise app
+(for company)</t>
+  </si>
+  <si>
+    <t>replit</t>
+  </si>
+  <si>
+    <t>Starter Monthly</t>
+  </si>
+  <si>
+    <t>Replit Core Monthly</t>
+  </si>
+  <si>
+    <t>Replit Pro Monthly</t>
+  </si>
+  <si>
+    <t>Enterprise Monthly</t>
+  </si>
+  <si>
+    <t>Starter Yearly</t>
+  </si>
+  <si>
+    <t>Replit Core Yearly</t>
+  </si>
+  <si>
+    <t>Replit Pro Yearly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://openai.com/index/introducing-gpt-5-4-mini-and-nano/
+</t>
+  </si>
+  <si>
+    <t>https://github.com/copilot
+https://docs.github.com/en/copilot/reference/ai-models/supported-models</t>
+  </si>
+  <si>
+    <t>gpt-5.4mini
+purpose or use case</t>
+  </si>
+  <si>
+    <t>gpt-5.4 nano 
+purpose or use case</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="[$$-409]#,##0.000"/>
     <numFmt numFmtId="167" formatCode="#,##0.000"/>
+    <numFmt numFmtId="172" formatCode="#,##0.00\ &quot;credits&quot;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -493,6 +548,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -511,10 +574,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -547,8 +611,19 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -827,7 +902,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V125"/>
+  <dimension ref="A1:V159"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1082,6 +1157,9 @@
         <f>PRODUCT(SUM(G12,I12),12)</f>
         <v>453.12</v>
       </c>
+      <c r="L12" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -1675,447 +1753,665 @@
         <v>2</v>
       </c>
     </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="G74" s="8"/>
+      <c r="K74" s="7"/>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>133</v>
+      </c>
+      <c r="E75" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B76" s="7"/>
+      <c r="L76" s="1"/>
+      <c r="M76" s="1"/>
+    </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+      <c r="E77" s="18">
+        <v>500</v>
+      </c>
+      <c r="F77" s="16">
+        <f>1700/95.79</f>
+        <v>17.747155235410794</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E78" s="18">
+        <v>1000</v>
+      </c>
+      <c r="F78" s="16">
+        <f>3400/95.79</f>
+        <v>35.494310470821588</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E79" s="18">
+        <v>1500</v>
+      </c>
+      <c r="F79" s="16">
+        <f>5100/95.79</f>
+        <v>53.241465706232383</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E80" s="18">
+        <v>2500</v>
+      </c>
+      <c r="F80" s="16">
+        <f>8500/95.79</f>
+        <v>88.735776177053964</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E81" s="18">
+        <v>5000</v>
+      </c>
+      <c r="F81" s="16">
+        <f>17000/95.79</f>
+        <v>177.47155235410793</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E82" s="18">
+        <v>10000</v>
+      </c>
+      <c r="F82" s="16">
+        <f>34000/95.79</f>
+        <v>354.94310470821586</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B83" s="7"/>
+      <c r="E83" s="18">
+        <v>250</v>
+      </c>
+      <c r="F83" s="16">
+        <f>F77/2</f>
+        <v>8.8735776177053971</v>
+      </c>
+      <c r="L83" s="1"/>
+      <c r="M83" s="1"/>
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+      <c r="E84" s="18">
+        <v>750</v>
+      </c>
+      <c r="F84" s="7"/>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E85" s="18"/>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E86" s="18"/>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E87" s="16"/>
+    </row>
+    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>109</v>
       </c>
-      <c r="C78" t="s">
+      <c r="C89" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="79" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A79" s="11" t="s">
+    <row r="90" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A90" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="B79" s="14">
+      <c r="B90" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="80" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A80" s="11" t="s">
+    <row r="91" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A91" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="B80" s="14">
+      <c r="B91" s="14">
         <v>0.5</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A81" s="11" t="s">
+    <row r="92" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A92" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="B81" s="14">
+      <c r="B92" s="14">
         <v>30</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A82" s="11" t="s">
+    <row r="93" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A93" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="B82" s="15">
+      <c r="B93" s="15">
         <v>105000</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A83" s="11" t="s">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A94" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="B83" s="15">
+      <c r="B94" s="15">
         <v>128000</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B84" s="14"/>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B85" s="14"/>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B86" s="14"/>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B87" s="14"/>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B95" s="14"/>
+    </row>
+    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B96" s="14"/>
+    </row>
+    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B97" s="14"/>
+    </row>
+    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B98" s="14"/>
+    </row>
+    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>9</v>
       </c>
-      <c r="E89" t="s">
+      <c r="E100" t="s">
         <v>89</v>
       </c>
-      <c r="F89" s="7">
-        <v>0</v>
-      </c>
-      <c r="G89" s="7"/>
-      <c r="I89">
-        <v>0</v>
-      </c>
-      <c r="J89" s="7">
-        <f>SUM(F89,I89)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E90" t="s">
+      <c r="F100" s="7">
+        <v>0</v>
+      </c>
+      <c r="G100" s="7"/>
+      <c r="I100">
+        <v>0</v>
+      </c>
+      <c r="J100" s="7">
+        <f>SUM(F100,I100)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E101" t="s">
         <v>90</v>
       </c>
-      <c r="F90" s="7">
+      <c r="F101" s="7">
         <f>399/95.79</f>
         <v>4.1653617287817095</v>
       </c>
-      <c r="G90" s="7"/>
-      <c r="I90">
-        <v>0</v>
-      </c>
-      <c r="J90" s="7">
-        <f>SUM(F90,I90)</f>
+      <c r="G101" s="7"/>
+      <c r="I101">
+        <v>0</v>
+      </c>
+      <c r="J101" s="7">
+        <f>SUM(F101,I101)</f>
         <v>4.1653617287817095</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E91" t="s">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E102" t="s">
         <v>91</v>
       </c>
-      <c r="F91" s="7"/>
-      <c r="G91" s="7">
+      <c r="F102" s="7"/>
+      <c r="G102" s="7">
         <f>4000/95.79</f>
         <v>41.75801231861363</v>
       </c>
-      <c r="I91">
-        <v>0</v>
-      </c>
-      <c r="K91" s="7">
-        <f>SUM(G91,I91)</f>
+      <c r="I102">
+        <v>0</v>
+      </c>
+      <c r="K102" s="7">
+        <f>SUM(G102,I102)</f>
         <v>41.75801231861363</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E92" t="s">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E103" t="s">
         <v>92</v>
       </c>
-      <c r="F92" s="7">
+      <c r="F103" s="7">
         <f>1950/95.79</f>
         <v>20.357031005324146</v>
       </c>
-      <c r="I92">
-        <v>0</v>
-      </c>
-      <c r="J92" s="7">
-        <f>SUM(F92,I92)</f>
+      <c r="I103">
+        <v>0</v>
+      </c>
+      <c r="J103" s="7">
+        <f>SUM(F103,I103)</f>
         <v>20.357031005324146</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E93" t="s">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E104" t="s">
         <v>93</v>
       </c>
-      <c r="F93" s="7"/>
-      <c r="G93" s="7">
+      <c r="F104" s="7"/>
+      <c r="G104" s="7">
         <f>19500/95.79</f>
         <v>203.57031005324146</v>
       </c>
-      <c r="I93">
-        <v>0</v>
-      </c>
-      <c r="K93" s="7">
-        <f>SUM(G93,I93)</f>
+      <c r="I104">
+        <v>0</v>
+      </c>
+      <c r="K104" s="7">
+        <f>SUM(G104,I104)</f>
         <v>203.57031005324146</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E94" t="s">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E105" t="s">
         <v>94</v>
       </c>
-      <c r="F94" s="7">
+      <c r="F105" s="7">
         <f>6500/95.79</f>
         <v>67.856770017747152</v>
       </c>
-      <c r="G94" s="7"/>
-      <c r="I94">
-        <v>0</v>
-      </c>
-      <c r="J94" s="7">
-        <f>SUM(F94,I94)</f>
+      <c r="G105" s="7"/>
+      <c r="I105">
+        <v>0</v>
+      </c>
+      <c r="J105" s="7">
+        <f>SUM(F105,I105)</f>
         <v>67.856770017747152</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E95" t="s">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E106" t="s">
         <v>95</v>
       </c>
-      <c r="G95" s="7">
+      <c r="G106" s="7">
         <f>6500/95.79</f>
         <v>67.856770017747152</v>
       </c>
-      <c r="I95">
-        <v>0</v>
-      </c>
-      <c r="K95" s="7">
-        <f>SUM(G95,I95)</f>
+      <c r="I106">
+        <v>0</v>
+      </c>
+      <c r="K106" s="7">
+        <f>SUM(G106,I106)</f>
         <v>67.856770017747152</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+    <row r="107" spans="1:13" s="17" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B107" s="7"/>
+      <c r="E107" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="F107" s="7">
+        <v>14</v>
+      </c>
+      <c r="G107" s="7"/>
+      <c r="K107" s="7"/>
+      <c r="L107" s="1">
+        <v>1</v>
+      </c>
+      <c r="M107" s="1"/>
+    </row>
+    <row r="108" spans="1:13" s="17" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B108" s="7"/>
+      <c r="E108" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="F108" s="7">
+        <v>21</v>
+      </c>
+      <c r="G108" s="7"/>
+      <c r="K108" s="7"/>
+      <c r="L108" s="1"/>
+      <c r="M108" s="1"/>
+    </row>
+    <row r="109" spans="1:13" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B109" s="7"/>
+      <c r="G109" s="7"/>
+      <c r="K109" s="7"/>
+      <c r="L109" s="1"/>
+      <c r="M109" s="1"/>
+    </row>
+    <row r="110" spans="1:13" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B110" s="7"/>
+      <c r="G110" s="7"/>
+      <c r="K110" s="7"/>
+      <c r="L110" s="1"/>
+      <c r="M110" s="1"/>
+    </row>
+    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
+    <row r="119" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
         <v>10</v>
       </c>
-      <c r="E104" t="s">
+      <c r="E119" t="s">
         <v>96</v>
       </c>
-      <c r="F104" s="7">
-        <v>0</v>
-      </c>
-      <c r="I104" s="7">
-        <f>F104*0.18</f>
-        <v>0</v>
-      </c>
-      <c r="J104" s="7">
-        <f>SUM(F104,I104)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E105" t="s">
+      <c r="F119" s="7">
+        <v>0</v>
+      </c>
+      <c r="I119" s="7">
+        <f>F119*0.18</f>
+        <v>0</v>
+      </c>
+      <c r="J119" s="7">
+        <f>SUM(F119,I119)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E120" t="s">
         <v>97</v>
       </c>
-      <c r="F105" s="7">
+      <c r="F120" s="7">
         <v>20</v>
       </c>
-      <c r="I105" s="7">
-        <f>F105*0.18</f>
+      <c r="I120" s="7">
+        <f>F120*0.18</f>
         <v>3.5999999999999996</v>
       </c>
-      <c r="J105" s="7">
-        <f>SUM(F105,I105)</f>
+      <c r="J120" s="7">
+        <f>SUM(F120,I120)</f>
         <v>23.6</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E106" t="s">
+    <row r="121" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E121" t="s">
         <v>98</v>
       </c>
-      <c r="F106" s="7">
+      <c r="F121" s="7">
         <v>200</v>
       </c>
-      <c r="I106" s="7">
-        <f>F106*0.18</f>
+      <c r="I121" s="7">
+        <f>F121*0.18</f>
         <v>36</v>
       </c>
-      <c r="J106" s="7">
-        <f>SUM(F106,I106)</f>
+      <c r="J121" s="7">
+        <f>SUM(F121,I121)</f>
         <v>236</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E107" t="s">
+    <row r="122" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E122" t="s">
         <v>99</v>
       </c>
-      <c r="F107" s="7">
+      <c r="F122" s="7">
         <v>40</v>
       </c>
-      <c r="I107" s="7">
-        <f>F107*0.18</f>
+      <c r="I122" s="7">
+        <f>F122*0.18</f>
         <v>7.1999999999999993</v>
       </c>
-      <c r="J107" s="7">
-        <f>PRODUCT(SUM(F107,I107),M107)</f>
+      <c r="J122" s="7">
+        <f>PRODUCT(SUM(F122,I122),M122)</f>
         <v>94.4</v>
       </c>
-      <c r="L107" s="1">
-        <v>1</v>
-      </c>
-      <c r="M107" s="1">
+      <c r="L122" s="1">
+        <v>1</v>
+      </c>
+      <c r="M122" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
         <v>12</v>
       </c>
-      <c r="E109" t="s">
+      <c r="E124" t="s">
         <v>100</v>
       </c>
-      <c r="F109" s="7">
-        <v>0</v>
-      </c>
-      <c r="I109">
-        <v>0</v>
-      </c>
-      <c r="J109" s="7">
-        <f>PRODUCT(SUM(F109,I109),L109)</f>
-        <v>0</v>
-      </c>
-      <c r="L109" s="1">
+      <c r="F124" s="7">
+        <v>0</v>
+      </c>
+      <c r="I124">
+        <v>0</v>
+      </c>
+      <c r="J124" s="7">
+        <f>PRODUCT(SUM(F124,I124),L124)</f>
+        <v>0</v>
+      </c>
+      <c r="L124" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E110" t="s">
+    <row r="125" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E125" t="s">
         <v>101</v>
       </c>
-      <c r="F110" s="7">
+      <c r="F125" s="7">
         <v>30</v>
       </c>
-      <c r="I110">
-        <v>0</v>
-      </c>
-      <c r="J110" s="7">
-        <f>PRODUCT(SUM(F110,I110),L110)</f>
+      <c r="I125">
+        <v>0</v>
+      </c>
+      <c r="J125" s="7">
+        <f>PRODUCT(SUM(F125,I125),L125)</f>
         <v>30</v>
       </c>
-      <c r="L110" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E111" t="s">
+      <c r="L125" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E126" t="s">
         <v>102</v>
       </c>
-      <c r="F111" s="7">
+      <c r="F126" s="7">
         <v>100</v>
       </c>
-      <c r="I111">
-        <v>0</v>
-      </c>
-      <c r="J111" s="7">
-        <f>PRODUCT(SUM(F111,I111),L111)</f>
+      <c r="I126">
+        <v>0</v>
+      </c>
+      <c r="J126" s="7">
+        <f>PRODUCT(SUM(F126,I126),L126)</f>
         <v>200</v>
       </c>
-      <c r="L111" s="1">
+      <c r="L126" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
+    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
         <v>11</v>
       </c>
-      <c r="E113" t="s">
+      <c r="E128" t="s">
         <v>103</v>
       </c>
-      <c r="F113" s="7">
+      <c r="F128" s="7">
         <f>700/95.79</f>
         <v>7.3076521557573857</v>
       </c>
-      <c r="G113" s="7"/>
-      <c r="I113">
-        <v>0</v>
-      </c>
-      <c r="J113" s="7">
-        <f>SUM(F113,I113)</f>
+      <c r="G128" s="7"/>
+      <c r="I128">
+        <v>0</v>
+      </c>
+      <c r="J128" s="7">
+        <f>SUM(F128,I128)</f>
         <v>7.3076521557573857</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E114" t="s">
+    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E129" t="s">
         <v>104</v>
       </c>
-      <c r="F114" s="7">
+      <c r="F129" s="7">
         <v>30</v>
       </c>
-      <c r="G114" s="7"/>
-      <c r="I114">
-        <v>0</v>
-      </c>
-      <c r="J114" s="7">
-        <f>SUM(F114,I114)</f>
+      <c r="G129" s="7"/>
+      <c r="I129">
+        <v>0</v>
+      </c>
+      <c r="J129" s="7">
+        <f>SUM(F129,I129)</f>
         <v>30</v>
       </c>
-      <c r="M114" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E115" t="s">
+      <c r="M129" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E130" t="s">
         <v>105</v>
       </c>
-      <c r="F115" s="7">
+      <c r="F130" s="7">
         <v>300</v>
       </c>
-      <c r="G115" s="7"/>
-      <c r="I115">
-        <v>0</v>
-      </c>
-      <c r="J115" s="7">
-        <f>SUM(F115,I115)</f>
+      <c r="G130" s="7"/>
+      <c r="I130">
+        <v>0</v>
+      </c>
+      <c r="J130" s="7">
+        <f>SUM(F130,I130)</f>
         <v>300</v>
       </c>
-      <c r="M115" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E116" t="s">
+      <c r="M130" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E131" t="s">
         <v>106</v>
       </c>
-      <c r="G116" s="7">
+      <c r="G131" s="7">
         <v>300</v>
       </c>
-      <c r="I116">
-        <v>0</v>
-      </c>
-      <c r="K116" s="7">
-        <f>PRODUCT(SUM(G116,I116),12)</f>
+      <c r="I131">
+        <v>0</v>
+      </c>
+      <c r="K131" s="7">
+        <f>PRODUCT(SUM(G131,I131),12)</f>
         <v>3600</v>
       </c>
-      <c r="M116" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E117" t="s">
+      <c r="M131" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E132" t="s">
         <v>107</v>
       </c>
-      <c r="G117" s="7">
+      <c r="G132" s="7">
         <v>3000</v>
       </c>
-      <c r="I117">
-        <v>0</v>
-      </c>
-      <c r="K117" s="7">
-        <f>PRODUCT(SUM(G117,I117),12)</f>
+      <c r="I132">
+        <v>0</v>
+      </c>
+      <c r="K132" s="7">
+        <f>PRODUCT(SUM(G132,I132),12)</f>
         <v>36000</v>
       </c>
-      <c r="M117" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
+      <c r="M132" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
+    <row r="139" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
         <v>41</v>
       </c>
-      <c r="D124" t="s">
+      <c r="D139" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="D125" t="s">
+    <row r="140" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D140" t="s">
         <v>43</v>
       </c>
     </row>
+    <row r="143" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>136</v>
+      </c>
+      <c r="E143" t="s">
+        <v>137</v>
+      </c>
+      <c r="F143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E144" t="s">
+        <v>138</v>
+      </c>
+      <c r="F144">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E145" t="s">
+        <v>139</v>
+      </c>
+      <c r="F145">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E146" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E147" t="s">
+        <v>141</v>
+      </c>
+      <c r="G147">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E148" t="s">
+        <v>142</v>
+      </c>
+      <c r="G148">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E149" t="s">
+        <v>143</v>
+      </c>
+      <c r="G149">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A153" s="11" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A154" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="C154" s="19" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>4</v>
+      </c>
+      <c r="C159" s="11" t="s">
+        <v>145</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="3">
+  <dataValidations count="3">
     <dataValidation operator="greaterThanOrEqual" showErrorMessage="1" promptTitle="Input value" prompt="For chatgpt business plan with monthly billing seats must be greater than 2" sqref="L72" xr:uid="{AB019136-2B35-41BF-AAE3-7F915B8E1897}"/>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M73:N73 M107:N107" xr:uid="{8F453106-93E4-43B4-9F00-8386506E300D}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M73:N74 M122:N122" xr:uid="{8F453106-93E4-43B4-9F00-8386506E300D}">
       <formula1>2</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="input data valid" prompt="for Chatgpt business plan, seat number must be &gt;=2" sqref="M72:N72" xr:uid="{C3EC9F79-5D8D-4E87-BF0C-5E945135986B}">
       <formula1>2</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="C154" r:id="rId1" xr:uid="{4A3B5888-76A5-4C31-B7DB-DF01EAE42F77}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs:adding links to pricing data
</commit_message>
<xml_diff>
--- a/pricing-comparison.xlsx
+++ b/pricing-comparison.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\projects\leak-AI-cost-detector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4834485-6CD0-4336-A480-26750146DB09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{209134E8-5DDE-42D8-B58B-1ECABFAB9720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -522,7 +522,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="[$$-409]#,##0.000"/>
     <numFmt numFmtId="167" formatCode="#,##0.000"/>
-    <numFmt numFmtId="172" formatCode="#,##0.00\ &quot;credits&quot;"/>
+    <numFmt numFmtId="168" formatCode="#,##0.00\ &quot;credits&quot;"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -615,7 +615,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">

</xml_diff>